<commit_message>
added assign other provider scripts
</commit_message>
<xml_diff>
--- a/pageobjects/testData/files/usersCredentials.xlsx
+++ b/pageobjects/testData/files/usersCredentials.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAB7A1BD-3D99-4F10-B2F1-F4E4BCB97DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="1425" windowWidth="17280" windowHeight="8880"/>
+    <workbookView xWindow="1428" yWindow="1428" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="userCredentials" sheetId="7" r:id="rId1"/>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>admin</t>
   </si>
@@ -98,9 +99,6 @@
     <t>managingProviderForStatusCheck</t>
   </si>
   <si>
-    <t>managingauto@yopmail.com</t>
-  </si>
-  <si>
     <t>otherProviderForStatusCheck</t>
   </si>
   <si>
@@ -110,20 +108,20 @@
     <t>providerLoginCrendentails</t>
   </si>
   <si>
-    <t>testprovider2may@yopmail.com</t>
-  </si>
-  <si>
     <t>otherProviderForProviderStatusCheck</t>
   </si>
   <si>
     <t>testautootherproviderFP@yopmail.com</t>
+  </si>
+  <si>
+    <t>managingautoprovider@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -508,18 +506,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.140625" customWidth="1"/>
-    <col min="2" max="2" width="78.5703125" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.109375" customWidth="1"/>
+    <col min="2" max="2" width="78.5546875" customWidth="1"/>
+    <col min="3" max="3" width="37.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -536,7 +534,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -547,7 +545,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -558,7 +556,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -569,7 +567,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -580,7 +578,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -591,7 +589,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -602,7 +600,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -613,7 +611,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -624,7 +622,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -635,45 +633,45 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
+      <c r="B13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>30</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -686,9 +684,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
New feature file created for tracker modules
</commit_message>
<xml_diff>
--- a/pageobjects/testData/files/usersCredentials.xlsx
+++ b/pageobjects/testData/files/usersCredentials.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBB23D3-E31C-434C-ABB8-9A920B3C5C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1428" yWindow="1428" windowWidth="17280" windowHeight="8628" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1425" yWindow="1425" windowWidth="17280" windowHeight="8625"/>
   </bookViews>
   <sheets>
     <sheet name="userCredentials" sheetId="7" r:id="rId1"/>
@@ -72,9 +71,6 @@
     <t>FHDCMobileLogin</t>
   </si>
   <si>
-    <t>testcaregiver2may@yopmail.com</t>
-  </si>
-  <si>
     <t>downloadFHDALink</t>
   </si>
   <si>
@@ -118,13 +114,16 @@
   </si>
   <si>
     <t>checkuser</t>
+  </si>
+  <si>
+    <t>caregiverautotest@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -508,18 +507,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.88671875" customWidth="1"/>
-    <col min="2" max="2" width="78.5546875" customWidth="1"/>
-    <col min="3" max="3" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.85546875" customWidth="1"/>
+    <col min="2" max="2" width="78.5703125" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -536,7 +535,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -547,7 +546,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -558,7 +557,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -569,18 +568,18 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -591,100 +590,100 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>27</v>
       </c>
-      <c r="B14" t="s">
-        <v>28</v>
-      </c>
       <c r="C14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -697,9 +696,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Ios featurs files added
</commit_message>
<xml_diff>
--- a/pageobjects/testData/files/usersCredentials.xlsx
+++ b/pageobjects/testData/files/usersCredentials.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9492A5A3-1F29-403D-AA93-5968BAE975D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1428" yWindow="1428" windowWidth="17280" windowHeight="8628" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1425" yWindow="1425" windowWidth="17280" windowHeight="8625"/>
   </bookViews>
   <sheets>
     <sheet name="userCredentials" sheetId="7" r:id="rId1"/>
@@ -72,9 +71,6 @@
     <t>FHDCMobileLogin</t>
   </si>
   <si>
-    <t>testcaregiver2may@yopmail.com</t>
-  </si>
-  <si>
     <t>downloadFHDALink</t>
   </si>
   <si>
@@ -118,13 +114,16 @@
   </si>
   <si>
     <t>otherautoproviderProv@yopmail.com</t>
+  </si>
+  <si>
+    <t>caregiverautotest@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,18 +508,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.88671875" customWidth="1"/>
-    <col min="2" max="2" width="78.5546875" customWidth="1"/>
-    <col min="3" max="3" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.85546875" customWidth="1"/>
+    <col min="2" max="2" width="78.5703125" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -537,7 +536,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -548,7 +547,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -559,7 +558,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -570,18 +569,18 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -592,100 +591,100 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>27</v>
-      </c>
       <c r="B14" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -698,9 +697,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added android medical records verification scripts
</commit_message>
<xml_diff>
--- a/pageobjects/testData/files/usersCredentials.xlsx
+++ b/pageobjects/testData/files/usersCredentials.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECA594B-D2DF-4E04-AA63-FD187FBB8C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="1524" windowWidth="17280" windowHeight="8628" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="1530" windowWidth="17280" windowHeight="8625"/>
   </bookViews>
   <sheets>
     <sheet name="userCredentials" sheetId="7" r:id="rId1"/>
@@ -126,8 +125,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -512,18 +511,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.88671875" customWidth="1"/>
-    <col min="2" max="2" width="78.5546875" customWidth="1"/>
-    <col min="3" max="3" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.85546875" customWidth="1"/>
+    <col min="2" max="2" width="78.5703125" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -540,7 +539,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -551,7 +550,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -562,7 +561,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -573,7 +572,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -584,7 +583,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -595,18 +594,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -617,7 +616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -628,7 +627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -639,7 +638,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -650,7 +649,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -661,7 +660,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -672,7 +671,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -683,7 +682,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -701,9 +700,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>